<commit_message>
chore: actualizar archivos base, plantillas de informe y Login
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentos base/base_1.xlsx
+++ b/Documentos base/base_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://quitoturismo365-my.sharepoint.com/personal/acasa_quito-turismo_gob_ec/Documents/Documentos/Desarrollo/Seguimiento_contrataciones/Documentos base/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{CD749712-33A4-4CA1-880B-578632C3F049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CAAD79F-E7CB-42BF-B4F8-782BFF0B039F}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{CD749712-33A4-4CA1-880B-578632C3F049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2084437C-2E07-4978-B913-E96103C3BEA4}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CF27BB3C-9C75-451E-B492-5C3FC5B283D4}"/>
+    <workbookView minimized="1" xWindow="2730" yWindow="2730" windowWidth="14415" windowHeight="8370" xr2:uid="{CF27BB3C-9C75-451E-B492-5C3FC5B283D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Matriz POA 2026" sheetId="1" r:id="rId1"/>
@@ -2219,6 +2219,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>

</xml_diff>